<commit_message>
Backup parser code updates
</commit_message>
<xml_diff>
--- a/Reference Documents/Merchant category mapping.xlsx
+++ b/Reference Documents/Merchant category mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\waccache\PN1PEPF000069CE\EXCELCNV\49e9f7f0-0e47-4a29-91cd-d22b829fc26f\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="146" documentId="8_{2EE984B8-BE7D-42A6-B46C-4DDEACA32909}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9E8B021-1AB8-4EF8-AFBD-6B40B212293B}"/>
+  <xr:revisionPtr revIDLastSave="222" documentId="8_{2EE984B8-BE7D-42A6-B46C-4DDEACA32909}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05043ECC-30AD-4E97-97AE-C13416E1891C}"/>
   <bookViews>
-    <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" firstSheet="1" activeTab="2" xr2:uid="{C92CC430-4B32-4796-8D62-416574D6DE36}"/>
+    <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" firstSheet="2" activeTab="2" xr2:uid="{C92CC430-4B32-4796-8D62-416574D6DE36}"/>
   </bookViews>
   <sheets>
     <sheet name="Merchant category mapping" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="239">
   <si>
     <t>Keyword Pattern</t>
   </si>
@@ -663,6 +663,72 @@
   </si>
   <si>
     <t>Airtel</t>
+  </si>
+  <si>
+    <t>Other Transaction Details</t>
+  </si>
+  <si>
+    <t> </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bank Of Baroda Rupay Credit Card </t>
+  </si>
+  <si>
+    <t>Smoke</t>
+  </si>
+  <si>
+    <t>BoB Uni Gold Card</t>
+  </si>
+  <si>
+    <t>Bank Of Baroda</t>
+  </si>
+  <si>
+    <t>BoB SB Account</t>
+  </si>
+  <si>
+    <t>#Refund</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Received from </t>
+  </si>
+  <si>
+    <t>Income</t>
+  </si>
+  <si>
+    <t>Refund</t>
+  </si>
+  <si>
+    <t>Mukesh</t>
+  </si>
+  <si>
+    <t>ravidasmukesh64@ybl on PhonePe</t>
+  </si>
+  <si>
+    <t>Rent</t>
+  </si>
+  <si>
+    <t>Abhay Singh</t>
+  </si>
+  <si>
+    <t>abhay.flyinheaven-1@okaxis on Google Pay</t>
+  </si>
+  <si>
+    <t>Tution Fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Money sent to </t>
+  </si>
+  <si>
+    <t>Misc.</t>
+  </si>
+  <si>
+    <t>Mobile contact transfer</t>
+  </si>
+  <si>
+    <t>Bank 2 Bank</t>
+  </si>
+  <si>
+    <t>PayTm Lite</t>
   </si>
   <si>
     <t>#🪙 Investment</t>
@@ -696,7 +762,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -842,8 +908,15 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1023,8 +1096,14 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="21">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -1278,6 +1357,30 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1323,7 +1426,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1341,8 +1444,23 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -3363,311 +3481,567 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91AF2A8D-08DB-402A-B65E-BCCAEF7E03A5}">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" customWidth="1"/>
-    <col min="7" max="7" width="16.28515625" customWidth="1"/>
+    <col min="3" max="3" width="30.7109375" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
+    <col min="7" max="7" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.42578125" customWidth="1"/>
+    <col min="9" max="9" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:10">
+      <c r="A1" s="20" t="s">
         <v>151</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="20" t="s">
         <v>148</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="D1" s="21" t="s">
+        <v>149</v>
+      </c>
+      <c r="E1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="14"/>
+      <c r="H1" s="25" t="s">
         <v>149</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="25" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:10">
       <c r="A2" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="G2" s="14"/>
+      <c r="H2" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="I2" s="23" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="22" t="s">
+        <v>209</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15" t="s">
+        <v>210</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>211</v>
+      </c>
+      <c r="G3" s="14"/>
+      <c r="H3" s="23" t="s">
+        <v>158</v>
+      </c>
+      <c r="I3" s="23" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="22"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="23" t="s">
+        <v>162</v>
+      </c>
+      <c r="I4" s="23" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="30.75">
+      <c r="A5" s="22" t="s">
+        <v>198</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>199</v>
+      </c>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="G5" s="14"/>
+      <c r="H5" s="23" t="s">
+        <v>210</v>
+      </c>
+      <c r="I5" s="23" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="22" t="s">
+        <v>198</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="C6" s="16"/>
+      <c r="D6" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="F6" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="G6" s="14"/>
+      <c r="H6" s="23" t="s">
+        <v>213</v>
+      </c>
+      <c r="I6" s="23" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" s="22" t="s">
+        <v>197</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" s="14"/>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" s="15" t="s">
+        <v>215</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>216</v>
+      </c>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>218</v>
+      </c>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" s="24" t="s">
+        <v>189</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="G9" s="19"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="19"/>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" s="22" t="s">
+        <v>187</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>188</v>
+      </c>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
+      <c r="J10" s="19"/>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="G11" s="14"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="19"/>
+    </row>
+    <row r="12" spans="1:10" ht="30.75">
+      <c r="A12" s="22" t="s">
+        <v>179</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>219</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>220</v>
+      </c>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>221</v>
+      </c>
+      <c r="G12" s="14"/>
+      <c r="H12" s="19"/>
+      <c r="I12" s="19"/>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="A13" s="22" t="s">
+        <v>179</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="F13" s="15" t="s">
+        <v>177</v>
+      </c>
+      <c r="G13" s="14"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="19"/>
+    </row>
+    <row r="14" spans="1:10" ht="30.75">
+      <c r="A14" s="22" t="s">
         <v>175</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="15" t="s">
+      <c r="B14" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>223</v>
+      </c>
+      <c r="D14" s="22"/>
+      <c r="E14" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>224</v>
+      </c>
+      <c r="G14" s="14"/>
+      <c r="H14" s="19"/>
+      <c r="I14" s="19"/>
+    </row>
+    <row r="15" spans="1:10" ht="30.75">
+      <c r="A15" s="22" t="s">
         <v>175</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="16" t="s">
+      <c r="B15" s="15" t="s">
+        <v>225</v>
+      </c>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>226</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>227</v>
+      </c>
+      <c r="G15" s="14"/>
+      <c r="H15" s="19"/>
+      <c r="I15" s="19"/>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="A16" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B16" s="15" t="s">
         <v>182</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C16" s="15"/>
+      <c r="D16" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="E16" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="1" t="s">
+      <c r="F16" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="G16" s="14"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="19"/>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B17" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C17" s="15"/>
+      <c r="D17" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="E17" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="15" t="s">
-        <v>187</v>
-      </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="15" t="s">
-        <v>189</v>
-      </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="15" t="s">
-        <v>191</v>
-      </c>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="15" t="s">
+      <c r="F17" s="15" t="s">
+        <v>229</v>
+      </c>
+      <c r="G17" s="14"/>
+      <c r="H17" s="19"/>
+      <c r="I17" s="19"/>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="22" t="s">
         <v>192</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B18" s="15" t="s">
         <v>193</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C18" s="15"/>
+      <c r="D18" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="E18" s="15" t="s">
         <v>194</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="F18" s="15" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="15" t="s">
+      <c r="G18" s="14"/>
+      <c r="H18" s="19"/>
+      <c r="I18" s="19"/>
+    </row>
+    <row r="19" spans="1:9" ht="30.75">
+      <c r="A19" s="22" t="s">
         <v>192</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B19" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="15" t="s">
-        <v>197</v>
-      </c>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" s="15" t="s">
-        <v>198</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" s="15" t="s">
-        <v>198</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="A15" s="15" t="s">
+      <c r="C19" s="15"/>
+      <c r="D19" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>226</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>227</v>
+      </c>
+      <c r="G19" s="14"/>
+      <c r="H19" s="19"/>
+      <c r="I19" s="19"/>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="22" t="s">
+        <v>201</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="F20" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="G20" s="14"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="19"/>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="22" t="s">
+        <v>203</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="F21" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="G21" s="14"/>
+      <c r="H21" s="19"/>
+      <c r="I21" s="19"/>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="22" t="s">
         <v>200</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B22" s="15" t="s">
         <v>152</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C22" s="15"/>
+      <c r="D22" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="E22" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="F22" s="15" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" s="15" t="s">
-        <v>201</v>
-      </c>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="15" t="s">
+      <c r="G22" s="14"/>
+      <c r="H22" s="19"/>
+      <c r="I22" s="19"/>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="22" t="s">
         <v>200</v>
       </c>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1" t="s">
+      <c r="B23" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="E23" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="F23" s="15" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" s="15" t="s">
-        <v>203</v>
-      </c>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="15" t="s">
+      <c r="G23" s="14"/>
+      <c r="H23" s="19"/>
+      <c r="I23" s="19"/>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="17" t="s">
         <v>204</v>
       </c>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1" t="s">
+      <c r="B24" s="18" t="s">
+        <v>209</v>
+      </c>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18" t="s">
+        <v>209</v>
+      </c>
+      <c r="E24" s="18" t="s">
         <v>205</v>
       </c>
-      <c r="D19" s="1"/>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
-      <c r="A21" s="13" t="s">
-        <v>208</v>
-      </c>
-      <c r="B21" t="s">
+      <c r="F24" s="18" t="s">
         <v>209</v>
       </c>
-      <c r="C21" t="s">
+      <c r="G24" s="14"/>
+      <c r="H24" s="19"/>
+      <c r="I24" s="19"/>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" s="17" t="s">
+        <v>230</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>231</v>
+      </c>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18" t="s">
+        <v>209</v>
+      </c>
+      <c r="E25" s="18" t="s">
         <v>172</v>
       </c>
-      <c r="D21" t="s">
-        <v>210</v>
-      </c>
+      <c r="F25" s="18" t="s">
+        <v>232</v>
+      </c>
+      <c r="G25" s="14"/>
+      <c r="H25" s="19"/>
+      <c r="I25" s="19"/>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" s="11"/>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F25">
+    <sortCondition ref="A2:A25"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3682,42 +4056,42 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>211</v>
+        <v>233</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>212</v>
+        <v>234</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>213</v>
+        <v>235</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>213</v>
+        <v>235</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>214</v>
+        <v>236</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>214</v>
+        <v>236</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>215</v>
+        <v>237</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>215</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>216</v>
+        <v>238</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>216</v>
+        <v>238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>